<commit_message>
Add drag-to-reorder for the web fallback's home list too
- Implement touch/pointer-based drag reordering in the vanilla-JS web version, matching the native app's per-device, per-group ordering behavior (no library, just Pointer Events)
- Fix a bug in the drop handler where the drag transform was cleared before measuring the dropped position, so the reorder always computed the item's original index and nothing visibly moved
- Update design docs and test specs to mark F21 as covering both platforms

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_UI.xlsx
+++ b/設計書/テスト仕様書_UI.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3248,6 +3248,43 @@
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="n"/>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Web版(わが家)</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>F21</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>ドラッグ＆ドロップでの並び替え</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>行左端のハンドルアイコンを指で押したまま動かし、離す</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>その端末の中で一覧の並び順が変わり、再読み込み後も同じ並びが維持される</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="n"/>
+      <c r="I76" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Skip the home-registration screen when a name-based rejoin already has a home saved
- Include the member's home location/radii in the join response when the join resolved to an existing member (name match)
- On the app, use that to restore the local geofence config and re-arm background monitoring immediately, then route straight to the Home tab instead of the registration screen
- New joins, and resumed members who never registered a home, still go through registration as before

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_UI.xlsx
+++ b/設計書/テスト仕様書_UI.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3507,6 +3507,43 @@
       <c r="H82" s="2" t="n"/>
       <c r="I82" s="2" t="n"/>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>招待コードで参加する画面</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>F2/F3</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>復帰時・自宅登録済みの場合の画面省略</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>以前このグループで自宅位置を登録済みの名前で、別の端末(再インストール後など)から参加する</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>招待コードと以前と同じ名前を入力して参加する</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>自宅の登録画面を経由せず、直接ホーム画面が表示される。バックグラウンドの自動判定も再登録される</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="n"/>
+      <c r="I83" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>